<commit_message>
bez literek osób towarzyszących
</commit_message>
<xml_diff>
--- a/app/templates/beach_protocol_template.xlsx
+++ b/app/templates/beach_protocol_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\radek\Desktop\Sędziowanie\PROTOKOŁY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51BE12F2-7065-47F3-BA6E-7E67DE95B139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BA75AF-1846-405C-89F3-C3BA06875DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{447D8A4E-A4E1-7249-8518-4A7488659659}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="64">
   <si>
     <t>PROTOKÓŁ ZAWODÓW</t>
   </si>
@@ -230,9 +230,6 @@
   </si>
   <si>
     <t>6m</t>
-  </si>
-  <si>
-    <t>C</t>
   </si>
 </sst>
 </file>
@@ -1248,6 +1245,153 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1257,23 +1401,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1284,18 +1419,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="20" fontId="10" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1320,140 +1443,14 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2444,15 +2441,15 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="H2" s="138" t="s">
+      <c r="H2" s="123" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="138"/>
-      <c r="J2" s="138"/>
-      <c r="K2" s="138"/>
-      <c r="L2" s="138"/>
-      <c r="M2" s="138"/>
-      <c r="N2" s="138"/>
+      <c r="I2" s="123"/>
+      <c r="J2" s="123"/>
+      <c r="K2" s="123"/>
+      <c r="L2" s="123"/>
+      <c r="M2" s="123"/>
+      <c r="N2" s="123"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C3" s="2"/>
@@ -2535,10 +2532,10 @@
         <v>9</v>
       </c>
       <c r="R6" s="2"/>
-      <c r="S6" s="139"/>
-      <c r="T6" s="140"/>
-      <c r="U6" s="140"/>
-      <c r="V6" s="141"/>
+      <c r="S6" s="101"/>
+      <c r="T6" s="102"/>
+      <c r="U6" s="102"/>
+      <c r="V6" s="103"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B7" s="8"/>
@@ -2564,10 +2561,10 @@
         <v>13</v>
       </c>
       <c r="R7" s="2"/>
-      <c r="S7" s="142"/>
-      <c r="T7" s="143"/>
-      <c r="U7" s="143"/>
-      <c r="V7" s="144"/>
+      <c r="S7" s="104"/>
+      <c r="T7" s="105"/>
+      <c r="U7" s="105"/>
+      <c r="V7" s="106"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B8" s="8"/>
@@ -2606,82 +2603,82 @@
       </c>
     </row>
     <row r="10" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="110"/>
-      <c r="C10" s="111"/>
-      <c r="D10" s="111"/>
-      <c r="E10" s="111"/>
-      <c r="F10" s="111"/>
-      <c r="G10" s="110"/>
-      <c r="H10" s="111"/>
-      <c r="I10" s="111"/>
-      <c r="J10" s="111"/>
-      <c r="K10" s="111"/>
-      <c r="L10" s="111"/>
-      <c r="M10" s="111"/>
-      <c r="N10" s="111"/>
-      <c r="O10" s="111"/>
-      <c r="P10" s="111"/>
-      <c r="Q10" s="112"/>
-      <c r="S10" s="147"/>
-      <c r="T10" s="148"/>
-      <c r="U10" s="148"/>
-      <c r="V10" s="149"/>
+      <c r="B10" s="107"/>
+      <c r="C10" s="108"/>
+      <c r="D10" s="108"/>
+      <c r="E10" s="108"/>
+      <c r="F10" s="108"/>
+      <c r="G10" s="107"/>
+      <c r="H10" s="108"/>
+      <c r="I10" s="108"/>
+      <c r="J10" s="108"/>
+      <c r="K10" s="108"/>
+      <c r="L10" s="108"/>
+      <c r="M10" s="108"/>
+      <c r="N10" s="108"/>
+      <c r="O10" s="108"/>
+      <c r="P10" s="108"/>
+      <c r="Q10" s="109"/>
+      <c r="S10" s="112"/>
+      <c r="T10" s="113"/>
+      <c r="U10" s="113"/>
+      <c r="V10" s="114"/>
     </row>
     <row r="11" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="145" t="s">
+      <c r="C11" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145" t="s">
+      <c r="D11" s="110"/>
+      <c r="E11" s="110"/>
+      <c r="F11" s="110" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145" t="s">
+      <c r="G11" s="110"/>
+      <c r="H11" s="110"/>
+      <c r="I11" s="110" t="s">
         <v>22</v>
       </c>
-      <c r="J11" s="145"/>
-      <c r="K11" s="145"/>
-      <c r="L11" s="145" t="s">
+      <c r="J11" s="110"/>
+      <c r="K11" s="110"/>
+      <c r="L11" s="110" t="s">
         <v>23</v>
       </c>
-      <c r="M11" s="145"/>
-      <c r="N11" s="146" t="s">
+      <c r="M11" s="110"/>
+      <c r="N11" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="O11" s="145"/>
-      <c r="P11" s="145"/>
-      <c r="Q11" s="145"/>
-      <c r="S11" s="150"/>
-      <c r="T11" s="151"/>
-      <c r="U11" s="151"/>
-      <c r="V11" s="152"/>
+      <c r="O11" s="110"/>
+      <c r="P11" s="110"/>
+      <c r="Q11" s="110"/>
+      <c r="S11" s="115"/>
+      <c r="T11" s="116"/>
+      <c r="U11" s="116"/>
+      <c r="V11" s="117"/>
     </row>
     <row r="12" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>
-      <c r="C12" s="156"/>
-      <c r="D12" s="111"/>
-      <c r="E12" s="112"/>
-      <c r="F12" s="157"/>
-      <c r="G12" s="111"/>
-      <c r="H12" s="112"/>
-      <c r="I12" s="110"/>
-      <c r="J12" s="111"/>
-      <c r="K12" s="112"/>
-      <c r="L12" s="110"/>
-      <c r="M12" s="112"/>
-      <c r="N12" s="110"/>
-      <c r="O12" s="111"/>
-      <c r="P12" s="111"/>
-      <c r="Q12" s="112"/>
-      <c r="S12" s="153"/>
-      <c r="T12" s="154"/>
-      <c r="U12" s="154"/>
-      <c r="V12" s="155"/>
+      <c r="C12" s="121"/>
+      <c r="D12" s="108"/>
+      <c r="E12" s="109"/>
+      <c r="F12" s="122"/>
+      <c r="G12" s="108"/>
+      <c r="H12" s="109"/>
+      <c r="I12" s="107"/>
+      <c r="J12" s="108"/>
+      <c r="K12" s="109"/>
+      <c r="L12" s="107"/>
+      <c r="M12" s="109"/>
+      <c r="N12" s="107"/>
+      <c r="O12" s="108"/>
+      <c r="P12" s="108"/>
+      <c r="Q12" s="109"/>
+      <c r="S12" s="118"/>
+      <c r="T12" s="119"/>
+      <c r="U12" s="119"/>
+      <c r="V12" s="120"/>
     </row>
     <row r="13" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2705,23 +2702,23 @@
         <v>29</v>
       </c>
       <c r="H14" s="4"/>
-      <c r="J14" s="106" t="s">
+      <c r="J14" s="152" t="s">
         <v>36</v>
       </c>
-      <c r="K14" s="107"/>
-      <c r="L14" s="107"/>
-      <c r="M14" s="107"/>
-      <c r="N14" s="107"/>
-      <c r="O14" s="108"/>
+      <c r="K14" s="153"/>
+      <c r="L14" s="153"/>
+      <c r="M14" s="153"/>
+      <c r="N14" s="153"/>
+      <c r="O14" s="154"/>
       <c r="P14" s="37"/>
-      <c r="Q14" s="106" t="s">
+      <c r="Q14" s="152" t="s">
         <v>37</v>
       </c>
-      <c r="R14" s="107"/>
-      <c r="S14" s="107"/>
-      <c r="T14" s="107"/>
-      <c r="U14" s="107"/>
-      <c r="V14" s="108"/>
+      <c r="R14" s="153"/>
+      <c r="S14" s="153"/>
+      <c r="T14" s="153"/>
+      <c r="U14" s="153"/>
+      <c r="V14" s="154"/>
     </row>
     <row r="15" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
@@ -3236,9 +3233,7 @@
       <c r="V30" s="48"/>
     </row>
     <row r="31" spans="1:22" ht="13.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="86" t="s">
-        <v>30</v>
-      </c>
+      <c r="A31" s="86"/>
       <c r="B31" s="84"/>
       <c r="C31" s="20"/>
       <c r="D31" s="91"/>
@@ -3269,9 +3264,7 @@
       <c r="V31" s="48"/>
     </row>
     <row r="32" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
-        <v>31</v>
-      </c>
+      <c r="A32" s="5"/>
       <c r="B32" s="82"/>
       <c r="C32" s="21"/>
       <c r="D32" s="93"/>
@@ -3302,9 +3295,7 @@
       <c r="V32" s="48"/>
     </row>
     <row r="33" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="87" t="s">
-        <v>64</v>
-      </c>
+      <c r="A33" s="87"/>
       <c r="B33" s="85"/>
       <c r="C33" s="16"/>
       <c r="D33" s="36"/>
@@ -3335,9 +3326,7 @@
       <c r="V33" s="48"/>
     </row>
     <row r="34" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="5" t="s">
-        <v>29</v>
-      </c>
+      <c r="A34" s="5"/>
       <c r="B34" s="82"/>
       <c r="C34" s="21"/>
       <c r="D34" s="93"/>
@@ -3373,11 +3362,11 @@
       </c>
       <c r="B35" s="34"/>
       <c r="C35" s="18"/>
-      <c r="D35" s="97" t="s">
+      <c r="D35" s="146" t="s">
         <v>33</v>
       </c>
-      <c r="E35" s="98"/>
-      <c r="F35" s="99"/>
+      <c r="E35" s="147"/>
+      <c r="F35" s="148"/>
       <c r="G35" s="95"/>
       <c r="H35" s="96"/>
       <c r="J35" s="44"/>
@@ -3849,16 +3838,16 @@
       <c r="J51" s="22"/>
       <c r="K51" s="23"/>
       <c r="L51" s="24"/>
-      <c r="M51" s="113"/>
-      <c r="N51" s="114"/>
-      <c r="O51" s="115"/>
+      <c r="M51" s="155"/>
+      <c r="N51" s="156"/>
+      <c r="O51" s="157"/>
       <c r="P51" s="23"/>
       <c r="Q51" s="25"/>
       <c r="R51" s="23"/>
       <c r="S51" s="24"/>
-      <c r="T51" s="113"/>
-      <c r="U51" s="114"/>
-      <c r="V51" s="119"/>
+      <c r="T51" s="155"/>
+      <c r="U51" s="156"/>
+      <c r="V51" s="161"/>
     </row>
     <row r="52" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5"/>
@@ -3873,16 +3862,16 @@
         <v>36</v>
       </c>
       <c r="L52" s="15"/>
-      <c r="M52" s="116"/>
-      <c r="N52" s="117"/>
-      <c r="O52" s="118"/>
+      <c r="M52" s="158"/>
+      <c r="N52" s="159"/>
+      <c r="O52" s="160"/>
       <c r="Q52" s="27" t="s">
         <v>37</v>
       </c>
       <c r="S52" s="15"/>
-      <c r="T52" s="116"/>
-      <c r="U52" s="117"/>
-      <c r="V52" s="120"/>
+      <c r="T52" s="158"/>
+      <c r="U52" s="159"/>
+      <c r="V52" s="162"/>
     </row>
     <row r="53" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="29"/>
@@ -3896,20 +3885,18 @@
       <c r="J53" s="30"/>
       <c r="K53" s="12"/>
       <c r="L53" s="12"/>
-      <c r="M53" s="100"/>
-      <c r="N53" s="121"/>
-      <c r="O53" s="122"/>
+      <c r="M53" s="124"/>
+      <c r="N53" s="125"/>
+      <c r="O53" s="163"/>
       <c r="Q53" s="11"/>
       <c r="R53" s="12"/>
       <c r="S53" s="13"/>
-      <c r="T53" s="100"/>
-      <c r="U53" s="121"/>
-      <c r="V53" s="101"/>
+      <c r="T53" s="124"/>
+      <c r="U53" s="125"/>
+      <c r="V53" s="126"/>
     </row>
     <row r="54" spans="1:22" ht="13.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="86" t="s">
-        <v>30</v>
-      </c>
+      <c r="A54" s="86"/>
       <c r="B54" s="84"/>
       <c r="C54" s="20"/>
       <c r="D54" s="91"/>
@@ -3920,21 +3907,19 @@
       <c r="J54" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="M54" s="102"/>
-      <c r="N54" s="123"/>
-      <c r="O54" s="124"/>
+      <c r="M54" s="127"/>
+      <c r="N54" s="128"/>
+      <c r="O54" s="164"/>
       <c r="Q54" s="27" t="s">
         <v>38</v>
       </c>
       <c r="S54" s="15"/>
-      <c r="T54" s="102"/>
-      <c r="U54" s="123"/>
-      <c r="V54" s="103"/>
+      <c r="T54" s="127"/>
+      <c r="U54" s="128"/>
+      <c r="V54" s="129"/>
     </row>
     <row r="55" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="5" t="s">
-        <v>31</v>
-      </c>
+      <c r="A55" s="5"/>
       <c r="B55" s="82"/>
       <c r="C55" s="21"/>
       <c r="D55" s="93"/>
@@ -3943,19 +3928,17 @@
       <c r="G55" s="89"/>
       <c r="H55" s="89"/>
       <c r="J55" s="32"/>
-      <c r="M55" s="104"/>
-      <c r="N55" s="125"/>
-      <c r="O55" s="126"/>
+      <c r="M55" s="130"/>
+      <c r="N55" s="131"/>
+      <c r="O55" s="165"/>
       <c r="Q55" s="14"/>
       <c r="S55" s="15"/>
-      <c r="T55" s="104"/>
-      <c r="U55" s="125"/>
-      <c r="V55" s="105"/>
+      <c r="T55" s="130"/>
+      <c r="U55" s="131"/>
+      <c r="V55" s="132"/>
     </row>
     <row r="56" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="87" t="s">
-        <v>64</v>
-      </c>
+      <c r="A56" s="87"/>
       <c r="B56" s="85"/>
       <c r="C56" s="16"/>
       <c r="D56" s="36"/>
@@ -3977,14 +3960,12 @@
       </c>
       <c r="R56" s="54"/>
       <c r="S56" s="55"/>
-      <c r="T56" s="133"/>
-      <c r="U56" s="134"/>
-      <c r="V56" s="135"/>
+      <c r="T56" s="139"/>
+      <c r="U56" s="140"/>
+      <c r="V56" s="141"/>
     </row>
     <row r="57" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="5" t="s">
-        <v>29</v>
-      </c>
+      <c r="A57" s="5"/>
       <c r="B57" s="82"/>
       <c r="C57" s="21"/>
       <c r="D57" s="93"/>
@@ -4004,22 +3985,22 @@
       <c r="Q57" s="59"/>
       <c r="R57" s="57"/>
       <c r="S57" s="58"/>
-      <c r="T57" s="127"/>
-      <c r="U57" s="128"/>
-      <c r="V57" s="129"/>
+      <c r="T57" s="133"/>
+      <c r="U57" s="134"/>
+      <c r="V57" s="135"/>
     </row>
     <row r="58" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="B58" s="158"/>
+      <c r="B58" s="97"/>
       <c r="C58" s="13"/>
-      <c r="D58" s="159" t="s">
+      <c r="D58" s="149" t="s">
         <v>33</v>
       </c>
-      <c r="E58" s="160"/>
-      <c r="F58" s="161"/>
-      <c r="G58" s="162"/>
+      <c r="E58" s="150"/>
+      <c r="F58" s="151"/>
+      <c r="G58" s="98"/>
       <c r="H58" s="90"/>
       <c r="I58" s="28"/>
       <c r="J58" s="60" t="s">
@@ -4036,19 +4017,19 @@
       </c>
       <c r="R58" s="64"/>
       <c r="S58" s="65"/>
-      <c r="T58" s="130"/>
-      <c r="U58" s="131"/>
-      <c r="V58" s="132"/>
+      <c r="T58" s="136"/>
+      <c r="U58" s="137"/>
+      <c r="V58" s="138"/>
     </row>
     <row r="59" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="163"/>
-      <c r="B59" s="164"/>
-      <c r="C59" s="165"/>
-      <c r="D59" s="165"/>
-      <c r="E59" s="165"/>
-      <c r="F59" s="165"/>
-      <c r="G59" s="165"/>
-      <c r="H59" s="165"/>
+      <c r="A59" s="99"/>
+      <c r="B59" s="100"/>
+      <c r="C59" s="142"/>
+      <c r="D59" s="142"/>
+      <c r="E59" s="142"/>
+      <c r="F59" s="142"/>
+      <c r="G59" s="142"/>
+      <c r="H59" s="142"/>
       <c r="J59" s="66" t="s">
         <v>34</v>
       </c>
@@ -4062,24 +4043,24 @@
       <c r="R59" s="72"/>
       <c r="S59" s="72"/>
       <c r="T59" s="72"/>
-      <c r="U59" s="100"/>
-      <c r="V59" s="101"/>
+      <c r="U59" s="124"/>
+      <c r="V59" s="126"/>
     </row>
     <row r="60" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="109" t="s">
+      <c r="A60" s="145" t="s">
         <v>44</v>
       </c>
-      <c r="B60" s="109"/>
-      <c r="C60" s="109" t="s">
+      <c r="B60" s="145"/>
+      <c r="C60" s="145" t="s">
         <v>45</v>
       </c>
-      <c r="D60" s="109"/>
-      <c r="E60" s="109"/>
-      <c r="F60" s="109" t="s">
+      <c r="D60" s="145"/>
+      <c r="E60" s="145"/>
+      <c r="F60" s="145" t="s">
         <v>46</v>
       </c>
-      <c r="G60" s="109"/>
-      <c r="H60" s="109"/>
+      <c r="G60" s="145"/>
+      <c r="H60" s="145"/>
       <c r="J60" s="67" t="s">
         <v>47</v>
       </c>
@@ -4093,20 +4074,20 @@
       <c r="R60" s="75"/>
       <c r="S60" s="75"/>
       <c r="T60" s="75"/>
-      <c r="U60" s="102"/>
-      <c r="V60" s="103"/>
+      <c r="U60" s="127"/>
+      <c r="V60" s="129"/>
     </row>
     <row r="61" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
         <v>1</v>
       </c>
       <c r="B61" s="82"/>
-      <c r="C61" s="110"/>
-      <c r="D61" s="111"/>
-      <c r="E61" s="112"/>
-      <c r="F61" s="111"/>
-      <c r="G61" s="111"/>
-      <c r="H61" s="112"/>
+      <c r="C61" s="107"/>
+      <c r="D61" s="108"/>
+      <c r="E61" s="109"/>
+      <c r="F61" s="108"/>
+      <c r="G61" s="108"/>
+      <c r="H61" s="109"/>
       <c r="J61" s="68" t="s">
         <v>63</v>
       </c>
@@ -4120,20 +4101,20 @@
       <c r="R61" s="75"/>
       <c r="S61" s="75"/>
       <c r="T61" s="75"/>
-      <c r="U61" s="102"/>
-      <c r="V61" s="103"/>
+      <c r="U61" s="127"/>
+      <c r="V61" s="129"/>
     </row>
     <row r="62" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
         <v>2</v>
       </c>
       <c r="B62" s="85"/>
-      <c r="C62" s="110"/>
-      <c r="D62" s="111"/>
-      <c r="E62" s="112"/>
-      <c r="F62" s="111"/>
-      <c r="G62" s="111"/>
-      <c r="H62" s="112"/>
+      <c r="C62" s="107"/>
+      <c r="D62" s="108"/>
+      <c r="E62" s="109"/>
+      <c r="F62" s="108"/>
+      <c r="G62" s="108"/>
+      <c r="H62" s="109"/>
       <c r="J62" s="67" t="s">
         <v>27</v>
       </c>
@@ -4147,8 +4128,8 @@
       <c r="R62" s="75"/>
       <c r="S62" s="75"/>
       <c r="T62" s="75"/>
-      <c r="U62" s="136"/>
-      <c r="V62" s="137"/>
+      <c r="U62" s="143"/>
+      <c r="V62" s="144"/>
     </row>
     <row r="63" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="1" t="s">
@@ -4175,12 +4156,12 @@
         <v>1</v>
       </c>
       <c r="B64" s="82"/>
-      <c r="C64" s="110"/>
-      <c r="D64" s="111"/>
-      <c r="E64" s="112"/>
-      <c r="F64" s="111"/>
-      <c r="G64" s="111"/>
-      <c r="H64" s="112"/>
+      <c r="C64" s="107"/>
+      <c r="D64" s="108"/>
+      <c r="E64" s="109"/>
+      <c r="F64" s="108"/>
+      <c r="G64" s="108"/>
+      <c r="H64" s="109"/>
       <c r="J64" s="67" t="s">
         <v>34</v>
       </c>
@@ -4194,20 +4175,20 @@
       <c r="R64" s="75"/>
       <c r="S64" s="75"/>
       <c r="T64" s="75"/>
-      <c r="U64" s="100"/>
-      <c r="V64" s="101"/>
+      <c r="U64" s="124"/>
+      <c r="V64" s="126"/>
     </row>
     <row r="65" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5">
         <v>2</v>
       </c>
       <c r="B65" s="85"/>
-      <c r="C65" s="110"/>
-      <c r="D65" s="111"/>
-      <c r="E65" s="112"/>
-      <c r="F65" s="111"/>
-      <c r="G65" s="111"/>
-      <c r="H65" s="112"/>
+      <c r="C65" s="107"/>
+      <c r="D65" s="108"/>
+      <c r="E65" s="109"/>
+      <c r="F65" s="108"/>
+      <c r="G65" s="108"/>
+      <c r="H65" s="109"/>
       <c r="J65" s="67" t="s">
         <v>47</v>
       </c>
@@ -4221,8 +4202,8 @@
       <c r="R65" s="75"/>
       <c r="S65" s="75"/>
       <c r="T65" s="75"/>
-      <c r="U65" s="102"/>
-      <c r="V65" s="103"/>
+      <c r="U65" s="127"/>
+      <c r="V65" s="129"/>
     </row>
     <row r="66" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="9" t="s">
@@ -4241,20 +4222,20 @@
       <c r="R66" s="75"/>
       <c r="S66" s="75"/>
       <c r="T66" s="75"/>
-      <c r="U66" s="102"/>
-      <c r="V66" s="103"/>
+      <c r="U66" s="127"/>
+      <c r="V66" s="129"/>
     </row>
     <row r="67" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5">
         <v>1</v>
       </c>
       <c r="B67" s="82"/>
-      <c r="C67" s="110"/>
-      <c r="D67" s="111"/>
-      <c r="E67" s="112"/>
-      <c r="F67" s="110"/>
-      <c r="G67" s="111"/>
-      <c r="H67" s="112"/>
+      <c r="C67" s="107"/>
+      <c r="D67" s="108"/>
+      <c r="E67" s="109"/>
+      <c r="F67" s="107"/>
+      <c r="G67" s="108"/>
+      <c r="H67" s="109"/>
       <c r="J67" s="70" t="s">
         <v>27</v>
       </c>
@@ -4268,8 +4249,8 @@
       <c r="R67" s="80"/>
       <c r="S67" s="80"/>
       <c r="T67" s="80"/>
-      <c r="U67" s="104"/>
-      <c r="V67" s="105"/>
+      <c r="U67" s="130"/>
+      <c r="V67" s="132"/>
     </row>
     <row r="68" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="69" spans="1:22" s="33" customFormat="1" ht="8.4" x14ac:dyDescent="0.2">
@@ -4331,6 +4312,34 @@
     <row r="71" spans="1:22" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="U64:V67"/>
+    <mergeCell ref="J14:O14"/>
+    <mergeCell ref="Q14:V14"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="F62:H62"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="F64:H64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="F65:H65"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="F67:H67"/>
+    <mergeCell ref="M51:O52"/>
+    <mergeCell ref="T51:V52"/>
+    <mergeCell ref="M53:O55"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="F60:H60"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="F61:H61"/>
+    <mergeCell ref="H2:N2"/>
+    <mergeCell ref="T53:V55"/>
+    <mergeCell ref="T57:V58"/>
+    <mergeCell ref="T56:V56"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="F59:H59"/>
+    <mergeCell ref="U59:V62"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="D58:F58"/>
     <mergeCell ref="S6:V7"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="G10:Q10"/>
@@ -4345,34 +4354,6 @@
     <mergeCell ref="I12:K12"/>
     <mergeCell ref="L12:M12"/>
     <mergeCell ref="N12:Q12"/>
-    <mergeCell ref="H2:N2"/>
-    <mergeCell ref="T53:V55"/>
-    <mergeCell ref="T57:V58"/>
-    <mergeCell ref="T56:V56"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="F59:H59"/>
-    <mergeCell ref="U59:V62"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="F60:H60"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="F61:H61"/>
-    <mergeCell ref="D35:F35"/>
-    <mergeCell ref="D58:F58"/>
-    <mergeCell ref="U64:V67"/>
-    <mergeCell ref="J14:O14"/>
-    <mergeCell ref="Q14:V14"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="F62:H62"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="F64:H64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="F65:H65"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="F67:H67"/>
-    <mergeCell ref="M51:O52"/>
-    <mergeCell ref="T51:V52"/>
-    <mergeCell ref="M53:O55"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.39370078740157483" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="81" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
poprawka 3. seta i podpisów
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/app/templates/beach_protocol_template.xlsx
+++ b/app/templates/beach_protocol_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\radek\Desktop\Sędziowanie\PROTOKOŁY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\radek\Desktop\BAZA_ALL\zprp-backend\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BA75AF-1846-405C-89F3-C3BA06875DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98138D4-5F80-46AB-9FC8-9A547979B161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{447D8A4E-A4E1-7249-8518-4A7488659659}"/>
+    <workbookView xWindow="3000" yWindow="3000" windowWidth="17280" windowHeight="9960" xr2:uid="{447D8A4E-A4E1-7249-8518-4A7488659659}"/>
   </bookViews>
   <sheets>
     <sheet name="BLANK" sheetId="2" r:id="rId1"/>
@@ -1047,7 +1047,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -1239,12 +1239,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1257,23 +1251,32 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1284,6 +1287,126 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1323,133 +1446,7 @@
     <xf numFmtId="20" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2441,15 +2438,15 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="H2" s="123" t="s">
+      <c r="H2" s="126" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="123"/>
-      <c r="J2" s="123"/>
-      <c r="K2" s="123"/>
-      <c r="L2" s="123"/>
-      <c r="M2" s="123"/>
-      <c r="N2" s="123"/>
+      <c r="I2" s="126"/>
+      <c r="J2" s="126"/>
+      <c r="K2" s="126"/>
+      <c r="L2" s="126"/>
+      <c r="M2" s="126"/>
+      <c r="N2" s="126"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C3" s="2"/>
@@ -2532,10 +2529,10 @@
         <v>9</v>
       </c>
       <c r="R6" s="2"/>
-      <c r="S6" s="101"/>
-      <c r="T6" s="102"/>
-      <c r="U6" s="102"/>
-      <c r="V6" s="103"/>
+      <c r="S6" s="145"/>
+      <c r="T6" s="146"/>
+      <c r="U6" s="146"/>
+      <c r="V6" s="147"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B7" s="8"/>
@@ -2561,10 +2558,10 @@
         <v>13</v>
       </c>
       <c r="R7" s="2"/>
-      <c r="S7" s="104"/>
-      <c r="T7" s="105"/>
-      <c r="U7" s="105"/>
-      <c r="V7" s="106"/>
+      <c r="S7" s="148"/>
+      <c r="T7" s="149"/>
+      <c r="U7" s="149"/>
+      <c r="V7" s="150"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B8" s="8"/>
@@ -2603,82 +2600,82 @@
       </c>
     </row>
     <row r="10" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="107"/>
-      <c r="C10" s="108"/>
-      <c r="D10" s="108"/>
-      <c r="E10" s="108"/>
-      <c r="F10" s="108"/>
-      <c r="G10" s="107"/>
-      <c r="H10" s="108"/>
-      <c r="I10" s="108"/>
-      <c r="J10" s="108"/>
-      <c r="K10" s="108"/>
-      <c r="L10" s="108"/>
-      <c r="M10" s="108"/>
-      <c r="N10" s="108"/>
-      <c r="O10" s="108"/>
-      <c r="P10" s="108"/>
-      <c r="Q10" s="109"/>
-      <c r="S10" s="112"/>
-      <c r="T10" s="113"/>
-      <c r="U10" s="113"/>
-      <c r="V10" s="114"/>
+      <c r="B10" s="108"/>
+      <c r="C10" s="109"/>
+      <c r="D10" s="109"/>
+      <c r="E10" s="109"/>
+      <c r="F10" s="109"/>
+      <c r="G10" s="108"/>
+      <c r="H10" s="109"/>
+      <c r="I10" s="109"/>
+      <c r="J10" s="109"/>
+      <c r="K10" s="109"/>
+      <c r="L10" s="109"/>
+      <c r="M10" s="109"/>
+      <c r="N10" s="109"/>
+      <c r="O10" s="109"/>
+      <c r="P10" s="109"/>
+      <c r="Q10" s="110"/>
+      <c r="S10" s="153"/>
+      <c r="T10" s="154"/>
+      <c r="U10" s="154"/>
+      <c r="V10" s="155"/>
     </row>
     <row r="11" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="110" t="s">
+      <c r="C11" s="151" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="110"/>
-      <c r="E11" s="110"/>
-      <c r="F11" s="110" t="s">
+      <c r="D11" s="151"/>
+      <c r="E11" s="151"/>
+      <c r="F11" s="151" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="110"/>
-      <c r="H11" s="110"/>
-      <c r="I11" s="110" t="s">
+      <c r="G11" s="151"/>
+      <c r="H11" s="151"/>
+      <c r="I11" s="151" t="s">
         <v>22</v>
       </c>
-      <c r="J11" s="110"/>
-      <c r="K11" s="110"/>
-      <c r="L11" s="110" t="s">
+      <c r="J11" s="151"/>
+      <c r="K11" s="151"/>
+      <c r="L11" s="151" t="s">
         <v>23</v>
       </c>
-      <c r="M11" s="110"/>
-      <c r="N11" s="111" t="s">
+      <c r="M11" s="151"/>
+      <c r="N11" s="152" t="s">
         <v>24</v>
       </c>
-      <c r="O11" s="110"/>
-      <c r="P11" s="110"/>
-      <c r="Q11" s="110"/>
-      <c r="S11" s="115"/>
-      <c r="T11" s="116"/>
-      <c r="U11" s="116"/>
-      <c r="V11" s="117"/>
+      <c r="O11" s="151"/>
+      <c r="P11" s="151"/>
+      <c r="Q11" s="151"/>
+      <c r="S11" s="156"/>
+      <c r="T11" s="157"/>
+      <c r="U11" s="157"/>
+      <c r="V11" s="158"/>
     </row>
     <row r="12" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>
-      <c r="C12" s="121"/>
-      <c r="D12" s="108"/>
-      <c r="E12" s="109"/>
-      <c r="F12" s="122"/>
-      <c r="G12" s="108"/>
-      <c r="H12" s="109"/>
-      <c r="I12" s="107"/>
-      <c r="J12" s="108"/>
-      <c r="K12" s="109"/>
-      <c r="L12" s="107"/>
-      <c r="M12" s="109"/>
-      <c r="N12" s="107"/>
-      <c r="O12" s="108"/>
-      <c r="P12" s="108"/>
-      <c r="Q12" s="109"/>
-      <c r="S12" s="118"/>
-      <c r="T12" s="119"/>
-      <c r="U12" s="119"/>
-      <c r="V12" s="120"/>
+      <c r="C12" s="162"/>
+      <c r="D12" s="109"/>
+      <c r="E12" s="110"/>
+      <c r="F12" s="163"/>
+      <c r="G12" s="109"/>
+      <c r="H12" s="110"/>
+      <c r="I12" s="108"/>
+      <c r="J12" s="109"/>
+      <c r="K12" s="110"/>
+      <c r="L12" s="108"/>
+      <c r="M12" s="110"/>
+      <c r="N12" s="108"/>
+      <c r="O12" s="109"/>
+      <c r="P12" s="109"/>
+      <c r="Q12" s="110"/>
+      <c r="S12" s="159"/>
+      <c r="T12" s="160"/>
+      <c r="U12" s="160"/>
+      <c r="V12" s="161"/>
     </row>
     <row r="13" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2702,23 +2699,23 @@
         <v>29</v>
       </c>
       <c r="H14" s="4"/>
-      <c r="J14" s="152" t="s">
+      <c r="J14" s="105" t="s">
         <v>36</v>
       </c>
-      <c r="K14" s="153"/>
-      <c r="L14" s="153"/>
-      <c r="M14" s="153"/>
-      <c r="N14" s="153"/>
-      <c r="O14" s="154"/>
+      <c r="K14" s="106"/>
+      <c r="L14" s="106"/>
+      <c r="M14" s="106"/>
+      <c r="N14" s="106"/>
+      <c r="O14" s="107"/>
       <c r="P14" s="37"/>
-      <c r="Q14" s="152" t="s">
+      <c r="Q14" s="105" t="s">
         <v>37</v>
       </c>
-      <c r="R14" s="153"/>
-      <c r="S14" s="153"/>
-      <c r="T14" s="153"/>
-      <c r="U14" s="153"/>
-      <c r="V14" s="154"/>
+      <c r="R14" s="106"/>
+      <c r="S14" s="106"/>
+      <c r="T14" s="106"/>
+      <c r="U14" s="106"/>
+      <c r="V14" s="107"/>
     </row>
     <row r="15" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
@@ -3362,13 +3359,13 @@
       </c>
       <c r="B35" s="34"/>
       <c r="C35" s="18"/>
-      <c r="D35" s="146" t="s">
+      <c r="D35" s="139" t="s">
         <v>33</v>
       </c>
-      <c r="E35" s="147"/>
-      <c r="F35" s="148"/>
-      <c r="G35" s="95"/>
-      <c r="H35" s="96"/>
+      <c r="E35" s="140"/>
+      <c r="F35" s="141"/>
+      <c r="G35" s="164"/>
+      <c r="H35" s="89"/>
       <c r="J35" s="44"/>
       <c r="K35" s="42">
         <v>20</v>
@@ -3838,16 +3835,16 @@
       <c r="J51" s="22"/>
       <c r="K51" s="23"/>
       <c r="L51" s="24"/>
-      <c r="M51" s="155"/>
-      <c r="N51" s="156"/>
-      <c r="O51" s="157"/>
+      <c r="M51" s="111"/>
+      <c r="N51" s="112"/>
+      <c r="O51" s="113"/>
       <c r="P51" s="23"/>
       <c r="Q51" s="25"/>
       <c r="R51" s="23"/>
       <c r="S51" s="24"/>
-      <c r="T51" s="155"/>
-      <c r="U51" s="156"/>
-      <c r="V51" s="161"/>
+      <c r="T51" s="111"/>
+      <c r="U51" s="112"/>
+      <c r="V51" s="117"/>
     </row>
     <row r="52" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5"/>
@@ -3862,16 +3859,16 @@
         <v>36</v>
       </c>
       <c r="L52" s="15"/>
-      <c r="M52" s="158"/>
-      <c r="N52" s="159"/>
-      <c r="O52" s="160"/>
+      <c r="M52" s="114"/>
+      <c r="N52" s="115"/>
+      <c r="O52" s="116"/>
       <c r="Q52" s="27" t="s">
         <v>37</v>
       </c>
       <c r="S52" s="15"/>
-      <c r="T52" s="158"/>
-      <c r="U52" s="159"/>
-      <c r="V52" s="162"/>
+      <c r="T52" s="114"/>
+      <c r="U52" s="115"/>
+      <c r="V52" s="118"/>
     </row>
     <row r="53" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="29"/>
@@ -3885,15 +3882,15 @@
       <c r="J53" s="30"/>
       <c r="K53" s="12"/>
       <c r="L53" s="12"/>
-      <c r="M53" s="124"/>
-      <c r="N53" s="125"/>
-      <c r="O53" s="163"/>
+      <c r="M53" s="99"/>
+      <c r="N53" s="119"/>
+      <c r="O53" s="120"/>
       <c r="Q53" s="11"/>
       <c r="R53" s="12"/>
       <c r="S53" s="13"/>
-      <c r="T53" s="124"/>
-      <c r="U53" s="125"/>
-      <c r="V53" s="126"/>
+      <c r="T53" s="99"/>
+      <c r="U53" s="119"/>
+      <c r="V53" s="100"/>
     </row>
     <row r="54" spans="1:22" ht="13.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A54" s="86"/>
@@ -3907,16 +3904,16 @@
       <c r="J54" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="M54" s="127"/>
-      <c r="N54" s="128"/>
-      <c r="O54" s="164"/>
+      <c r="M54" s="101"/>
+      <c r="N54" s="121"/>
+      <c r="O54" s="122"/>
       <c r="Q54" s="27" t="s">
         <v>38</v>
       </c>
       <c r="S54" s="15"/>
-      <c r="T54" s="127"/>
-      <c r="U54" s="128"/>
-      <c r="V54" s="129"/>
+      <c r="T54" s="101"/>
+      <c r="U54" s="121"/>
+      <c r="V54" s="102"/>
     </row>
     <row r="55" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5"/>
@@ -3928,14 +3925,14 @@
       <c r="G55" s="89"/>
       <c r="H55" s="89"/>
       <c r="J55" s="32"/>
-      <c r="M55" s="130"/>
-      <c r="N55" s="131"/>
-      <c r="O55" s="165"/>
+      <c r="M55" s="103"/>
+      <c r="N55" s="123"/>
+      <c r="O55" s="124"/>
       <c r="Q55" s="14"/>
       <c r="S55" s="15"/>
-      <c r="T55" s="130"/>
-      <c r="U55" s="131"/>
-      <c r="V55" s="132"/>
+      <c r="T55" s="103"/>
+      <c r="U55" s="123"/>
+      <c r="V55" s="104"/>
     </row>
     <row r="56" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="87"/>
@@ -3960,9 +3957,9 @@
       </c>
       <c r="R56" s="54"/>
       <c r="S56" s="55"/>
-      <c r="T56" s="139"/>
-      <c r="U56" s="140"/>
-      <c r="V56" s="141"/>
+      <c r="T56" s="133"/>
+      <c r="U56" s="134"/>
+      <c r="V56" s="135"/>
     </row>
     <row r="57" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5"/>
@@ -3985,22 +3982,22 @@
       <c r="Q57" s="59"/>
       <c r="R57" s="57"/>
       <c r="S57" s="58"/>
-      <c r="T57" s="133"/>
-      <c r="U57" s="134"/>
-      <c r="V57" s="135"/>
+      <c r="T57" s="127"/>
+      <c r="U57" s="128"/>
+      <c r="V57" s="129"/>
     </row>
     <row r="58" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="B58" s="97"/>
+      <c r="B58" s="95"/>
       <c r="C58" s="13"/>
-      <c r="D58" s="149" t="s">
+      <c r="D58" s="142" t="s">
         <v>33</v>
       </c>
-      <c r="E58" s="150"/>
-      <c r="F58" s="151"/>
-      <c r="G58" s="98"/>
+      <c r="E58" s="143"/>
+      <c r="F58" s="144"/>
+      <c r="G58" s="96"/>
       <c r="H58" s="90"/>
       <c r="I58" s="28"/>
       <c r="J58" s="60" t="s">
@@ -4017,19 +4014,19 @@
       </c>
       <c r="R58" s="64"/>
       <c r="S58" s="65"/>
-      <c r="T58" s="136"/>
-      <c r="U58" s="137"/>
-      <c r="V58" s="138"/>
+      <c r="T58" s="130"/>
+      <c r="U58" s="131"/>
+      <c r="V58" s="132"/>
     </row>
     <row r="59" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="99"/>
-      <c r="B59" s="100"/>
-      <c r="C59" s="142"/>
-      <c r="D59" s="142"/>
-      <c r="E59" s="142"/>
-      <c r="F59" s="142"/>
-      <c r="G59" s="142"/>
-      <c r="H59" s="142"/>
+      <c r="A59" s="97"/>
+      <c r="B59" s="98"/>
+      <c r="C59" s="136"/>
+      <c r="D59" s="136"/>
+      <c r="E59" s="136"/>
+      <c r="F59" s="136"/>
+      <c r="G59" s="136"/>
+      <c r="H59" s="136"/>
       <c r="J59" s="66" t="s">
         <v>34</v>
       </c>
@@ -4043,24 +4040,24 @@
       <c r="R59" s="72"/>
       <c r="S59" s="72"/>
       <c r="T59" s="72"/>
-      <c r="U59" s="124"/>
-      <c r="V59" s="126"/>
+      <c r="U59" s="99"/>
+      <c r="V59" s="100"/>
     </row>
     <row r="60" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="145" t="s">
+      <c r="A60" s="125" t="s">
         <v>44</v>
       </c>
-      <c r="B60" s="145"/>
-      <c r="C60" s="145" t="s">
+      <c r="B60" s="125"/>
+      <c r="C60" s="125" t="s">
         <v>45</v>
       </c>
-      <c r="D60" s="145"/>
-      <c r="E60" s="145"/>
-      <c r="F60" s="145" t="s">
+      <c r="D60" s="125"/>
+      <c r="E60" s="125"/>
+      <c r="F60" s="125" t="s">
         <v>46</v>
       </c>
-      <c r="G60" s="145"/>
-      <c r="H60" s="145"/>
+      <c r="G60" s="125"/>
+      <c r="H60" s="125"/>
       <c r="J60" s="67" t="s">
         <v>47</v>
       </c>
@@ -4074,20 +4071,20 @@
       <c r="R60" s="75"/>
       <c r="S60" s="75"/>
       <c r="T60" s="75"/>
-      <c r="U60" s="127"/>
-      <c r="V60" s="129"/>
+      <c r="U60" s="101"/>
+      <c r="V60" s="102"/>
     </row>
     <row r="61" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
         <v>1</v>
       </c>
       <c r="B61" s="82"/>
-      <c r="C61" s="107"/>
-      <c r="D61" s="108"/>
-      <c r="E61" s="109"/>
-      <c r="F61" s="108"/>
-      <c r="G61" s="108"/>
-      <c r="H61" s="109"/>
+      <c r="C61" s="108"/>
+      <c r="D61" s="109"/>
+      <c r="E61" s="110"/>
+      <c r="F61" s="109"/>
+      <c r="G61" s="109"/>
+      <c r="H61" s="110"/>
       <c r="J61" s="68" t="s">
         <v>63</v>
       </c>
@@ -4101,20 +4098,20 @@
       <c r="R61" s="75"/>
       <c r="S61" s="75"/>
       <c r="T61" s="75"/>
-      <c r="U61" s="127"/>
-      <c r="V61" s="129"/>
+      <c r="U61" s="101"/>
+      <c r="V61" s="102"/>
     </row>
     <row r="62" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
         <v>2</v>
       </c>
       <c r="B62" s="85"/>
-      <c r="C62" s="107"/>
-      <c r="D62" s="108"/>
-      <c r="E62" s="109"/>
-      <c r="F62" s="108"/>
-      <c r="G62" s="108"/>
-      <c r="H62" s="109"/>
+      <c r="C62" s="108"/>
+      <c r="D62" s="109"/>
+      <c r="E62" s="110"/>
+      <c r="F62" s="109"/>
+      <c r="G62" s="109"/>
+      <c r="H62" s="110"/>
       <c r="J62" s="67" t="s">
         <v>27</v>
       </c>
@@ -4128,8 +4125,8 @@
       <c r="R62" s="75"/>
       <c r="S62" s="75"/>
       <c r="T62" s="75"/>
-      <c r="U62" s="143"/>
-      <c r="V62" s="144"/>
+      <c r="U62" s="137"/>
+      <c r="V62" s="138"/>
     </row>
     <row r="63" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="1" t="s">
@@ -4156,12 +4153,12 @@
         <v>1</v>
       </c>
       <c r="B64" s="82"/>
-      <c r="C64" s="107"/>
-      <c r="D64" s="108"/>
-      <c r="E64" s="109"/>
-      <c r="F64" s="108"/>
-      <c r="G64" s="108"/>
-      <c r="H64" s="109"/>
+      <c r="C64" s="108"/>
+      <c r="D64" s="109"/>
+      <c r="E64" s="110"/>
+      <c r="F64" s="109"/>
+      <c r="G64" s="109"/>
+      <c r="H64" s="110"/>
       <c r="J64" s="67" t="s">
         <v>34</v>
       </c>
@@ -4175,20 +4172,20 @@
       <c r="R64" s="75"/>
       <c r="S64" s="75"/>
       <c r="T64" s="75"/>
-      <c r="U64" s="124"/>
-      <c r="V64" s="126"/>
+      <c r="U64" s="99"/>
+      <c r="V64" s="100"/>
     </row>
     <row r="65" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5">
         <v>2</v>
       </c>
       <c r="B65" s="85"/>
-      <c r="C65" s="107"/>
-      <c r="D65" s="108"/>
-      <c r="E65" s="109"/>
-      <c r="F65" s="108"/>
-      <c r="G65" s="108"/>
-      <c r="H65" s="109"/>
+      <c r="C65" s="108"/>
+      <c r="D65" s="109"/>
+      <c r="E65" s="110"/>
+      <c r="F65" s="109"/>
+      <c r="G65" s="109"/>
+      <c r="H65" s="110"/>
       <c r="J65" s="67" t="s">
         <v>47</v>
       </c>
@@ -4202,8 +4199,8 @@
       <c r="R65" s="75"/>
       <c r="S65" s="75"/>
       <c r="T65" s="75"/>
-      <c r="U65" s="127"/>
-      <c r="V65" s="129"/>
+      <c r="U65" s="101"/>
+      <c r="V65" s="102"/>
     </row>
     <row r="66" spans="1:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="9" t="s">
@@ -4222,20 +4219,20 @@
       <c r="R66" s="75"/>
       <c r="S66" s="75"/>
       <c r="T66" s="75"/>
-      <c r="U66" s="127"/>
-      <c r="V66" s="129"/>
+      <c r="U66" s="101"/>
+      <c r="V66" s="102"/>
     </row>
     <row r="67" spans="1:22" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5">
         <v>1</v>
       </c>
       <c r="B67" s="82"/>
-      <c r="C67" s="107"/>
-      <c r="D67" s="108"/>
-      <c r="E67" s="109"/>
-      <c r="F67" s="107"/>
-      <c r="G67" s="108"/>
-      <c r="H67" s="109"/>
+      <c r="C67" s="108"/>
+      <c r="D67" s="109"/>
+      <c r="E67" s="110"/>
+      <c r="F67" s="108"/>
+      <c r="G67" s="109"/>
+      <c r="H67" s="110"/>
       <c r="J67" s="70" t="s">
         <v>27</v>
       </c>
@@ -4249,8 +4246,8 @@
       <c r="R67" s="80"/>
       <c r="S67" s="80"/>
       <c r="T67" s="80"/>
-      <c r="U67" s="130"/>
-      <c r="V67" s="132"/>
+      <c r="U67" s="103"/>
+      <c r="V67" s="104"/>
     </row>
     <row r="68" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="69" spans="1:22" s="33" customFormat="1" ht="8.4" x14ac:dyDescent="0.2">
@@ -4312,25 +4309,13 @@
     <row r="71" spans="1:22" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="U64:V67"/>
-    <mergeCell ref="J14:O14"/>
-    <mergeCell ref="Q14:V14"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="F62:H62"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="F64:H64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="F65:H65"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="F67:H67"/>
-    <mergeCell ref="M51:O52"/>
-    <mergeCell ref="T51:V52"/>
-    <mergeCell ref="M53:O55"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="F60:H60"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="F61:H61"/>
+    <mergeCell ref="N11:Q11"/>
+    <mergeCell ref="S10:V12"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="F12:H12"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="N12:Q12"/>
     <mergeCell ref="H2:N2"/>
     <mergeCell ref="T53:V55"/>
     <mergeCell ref="T57:V58"/>
@@ -4347,13 +4332,25 @@
     <mergeCell ref="F11:H11"/>
     <mergeCell ref="I11:K11"/>
     <mergeCell ref="L11:M11"/>
-    <mergeCell ref="N11:Q11"/>
-    <mergeCell ref="S10:V12"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="F12:H12"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="N12:Q12"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="F60:H60"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="F61:H61"/>
+    <mergeCell ref="U64:V67"/>
+    <mergeCell ref="J14:O14"/>
+    <mergeCell ref="Q14:V14"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="F62:H62"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="F64:H64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="F65:H65"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="F67:H67"/>
+    <mergeCell ref="M51:O52"/>
+    <mergeCell ref="T51:V52"/>
+    <mergeCell ref="M53:O55"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.39370078740157483" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="81" orientation="portrait" r:id="rId1"/>

</xml_diff>